<commit_message>
Make grammar items compulsory
</commit_message>
<xml_diff>
--- a/inst/formr/bvq-1.0.3/bvq_grammar_catalan.xlsx
+++ b/inst/formr/bvq-1.0.3/bvq_grammar_catalan.xlsx
@@ -140,7 +140,7 @@
 For example ‘Mama llibre’, ‘Bebé jugar’, ‘això allà’")))`</t>
   </si>
   <si>
-    <t xml:space="preserve">*</t>
+    <t xml:space="preserve">!</t>
   </si>
   <si>
     <t xml:space="preserve">answer_below_label </t>
@@ -879,44 +879,48 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1113,7 +1117,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="20.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.65625" defaultRowHeight="20.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="53.5"/>
@@ -1259,14 +1263,11 @@
       <c r="C7" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="5" t="n">
-        <v>1</v>
-      </c>
       <c r="I7" s="5" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="8" s="5" customFormat="true" ht="55.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" s="5" customFormat="true" ht="52.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
         <v>12</v>
       </c>
@@ -1286,7 +1287,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" s="5" customFormat="true" ht="55.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" s="5" customFormat="true" ht="52.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
         <v>12</v>
       </c>
@@ -1306,7 +1307,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" s="5" customFormat="true" ht="55.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" s="5" customFormat="true" ht="52.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
         <v>12</v>
       </c>
@@ -1326,7 +1327,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" s="5" customFormat="true" ht="55.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" s="5" customFormat="true" ht="52.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>12</v>
       </c>
@@ -1346,7 +1347,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" s="5" customFormat="true" ht="55.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" s="5" customFormat="true" ht="52.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
         <v>35</v>
       </c>
@@ -1379,9 +1380,6 @@
       <c r="C13" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="5" t="n">
-        <v>1</v>
-      </c>
       <c r="E13" s="1"/>
       <c r="F13" s="1" t="s">
         <v>41</v>
@@ -1390,7 +1388,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" s="5" customFormat="true" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" s="5" customFormat="true" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
         <v>42</v>
       </c>
@@ -1411,7 +1409,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" s="5" customFormat="true" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" s="5" customFormat="true" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
         <v>45</v>
       </c>
@@ -1432,7 +1430,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" s="5" customFormat="true" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" s="5" customFormat="true" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
         <v>47</v>
       </c>
@@ -1453,7 +1451,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" s="5" customFormat="true" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" s="5" customFormat="true" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
         <v>49</v>
       </c>
@@ -1474,7 +1472,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" s="5" customFormat="true" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" s="5" customFormat="true" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
         <v>51</v>
       </c>
@@ -1495,7 +1493,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" s="5" customFormat="true" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" s="5" customFormat="true" ht="35.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
         <v>53</v>
       </c>
@@ -1549,193 +1547,193 @@
   <dimension ref="A1:C17"/>
   <sheetFormatPr defaultColWidth="20" defaultRowHeight="20.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="9" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="9" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="9" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="9" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="9" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="9" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="9" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="9" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="9" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="9" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="9" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="9" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="9" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="9" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="9" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="9" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1759,95 +1757,95 @@
   <sheetFormatPr defaultColWidth="20" defaultRowHeight="20.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="10" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="9" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="9" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="9" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>